<commit_message>
balance the module PLS folds and tell the README the bout response tracks growth
</commit_message>
<xml_diff>
--- a/02_HRvLR/08_Module_Detail/c_data/module_detail.xlsx
+++ b/02_HRvLR/08_Module_Detail/c_data/module_detail.xlsx
@@ -90837,16 +90837,16 @@
         <v>3794</v>
       </c>
       <c r="E2">
-        <v>0.171875</v>
+        <v>0.271875</v>
       </c>
       <c r="F2">
-        <v>0.421875</v>
+        <v>0.484375</v>
       </c>
       <c r="G2">
-        <v>0.78125</v>
+        <v>0.7734375</v>
       </c>
       <c r="H2">
-        <v>0.8651348651348651</v>
+        <v>0.8931068931068931</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -90863,16 +90863,16 @@
         <v>3794</v>
       </c>
       <c r="E3">
-        <v>0.390625</v>
+        <v>0.55625</v>
       </c>
       <c r="F3">
-        <v>0.421875</v>
+        <v>0.5</v>
       </c>
       <c r="G3">
-        <v>0.75</v>
+        <v>0.7890625</v>
       </c>
       <c r="H3">
-        <v>0.5744255744255744</v>
+        <v>0.3586413586413587</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -90889,16 +90889,16 @@
         <v>3794</v>
       </c>
       <c r="E4">
-        <v>0.546875</v>
+        <v>0.590625</v>
       </c>
       <c r="F4">
-        <v>0.4140625</v>
+        <v>0.484375</v>
       </c>
       <c r="G4">
-        <v>0.75</v>
+        <v>0.78125</v>
       </c>
       <c r="H4">
-        <v>0.2887112887112887</v>
+        <v>0.2657342657342657</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -90915,16 +90915,16 @@
         <v>3797</v>
       </c>
       <c r="E5">
-        <v>-0.5251794335941857</v>
+        <v>-0.6418680301132275</v>
       </c>
       <c r="F5">
-        <v>-0.2933062864859017</v>
+        <v>-0.3633815984780215</v>
       </c>
       <c r="G5">
-        <v>0.2713113495165034</v>
+        <v>0.2037008234755296</v>
       </c>
       <c r="H5">
-        <v>0.7062937062937062</v>
+        <v>0.7342657342657343</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -90941,16 +90941,16 @@
         <v>3797</v>
       </c>
       <c r="E6">
-        <v>-0.3182412980996894</v>
+        <v>-0.2664354060093331</v>
       </c>
       <c r="F6">
-        <v>-0.2965055062439163</v>
+        <v>-0.3797567626564622</v>
       </c>
       <c r="G6">
-        <v>0.2340939392530419</v>
+        <v>0.1575873513940882</v>
       </c>
       <c r="H6">
-        <v>0.5264735264735265</v>
+        <v>0.3916083916083916</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -90967,16 +90967,16 @@
         <v>3797</v>
       </c>
       <c r="E7">
-        <v>-0.6012534994459553</v>
+        <v>-0.597321159258056</v>
       </c>
       <c r="F7">
-        <v>-0.3233843516884358</v>
+        <v>-0.3636443313841438</v>
       </c>
       <c r="G7">
-        <v>0.2351386284656306</v>
+        <v>0.1757551795192376</v>
       </c>
       <c r="H7">
-        <v>0.7712287712287712</v>
+        <v>0.7092907092907093</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -90993,16 +90993,16 @@
         <v>3797</v>
       </c>
       <c r="E8">
-        <v>-0.4076233340407556</v>
+        <v>-0.5424852908153299</v>
       </c>
       <c r="F8">
-        <v>-0.2917689084850487</v>
+        <v>-0.36874872320336</v>
       </c>
       <c r="G8">
-        <v>0.2444283660723195</v>
+        <v>0.1854988758783541</v>
       </c>
       <c r="H8">
-        <v>0.6163836163836164</v>
+        <v>0.6583416583416584</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -91019,16 +91019,16 @@
         <v>3797</v>
       </c>
       <c r="E9">
-        <v>-0.140379813575138</v>
+        <v>-0.1755517282571608</v>
       </c>
       <c r="F9">
-        <v>-0.3095335301650277</v>
+        <v>-0.3436304728633033</v>
       </c>
       <c r="G9">
-        <v>0.2777046854689</v>
+        <v>0.1832098444098669</v>
       </c>
       <c r="H9">
-        <v>0.3316683316683317</v>
+        <v>0.3196803196803197</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -91045,16 +91045,16 @@
         <v>3797</v>
       </c>
       <c r="E10">
-        <v>0.1335615512239963</v>
+        <v>0.05947687514625981</v>
       </c>
       <c r="F10">
-        <v>-0.2820748957833125</v>
+        <v>-0.3861372804742562</v>
       </c>
       <c r="G10">
-        <v>0.2084216063381978</v>
+        <v>0.1575690418699169</v>
       </c>
       <c r="H10">
-        <v>0.0899100899100899</v>
+        <v>0.0979020979020979</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -91071,16 +91071,16 @@
         <v>3797</v>
       </c>
       <c r="E11">
-        <v>-0.2435287968761048</v>
+        <v>-0.1630782764293885</v>
       </c>
       <c r="F11">
-        <v>-0.3039642795632621</v>
+        <v>-0.3735434548394063</v>
       </c>
       <c r="G11">
-        <v>0.2134926374684122</v>
+        <v>0.164485253501656</v>
       </c>
       <c r="H11">
-        <v>0.4265734265734266</v>
+        <v>0.2787212787212787</v>
       </c>
     </row>
     <row r="12" spans="1:8">
@@ -91097,16 +91097,16 @@
         <v>3797</v>
       </c>
       <c r="E12">
-        <v>-0.1777512182065355</v>
+        <v>-0.4054390463402516</v>
       </c>
       <c r="F12">
-        <v>-0.3020610330156486</v>
+        <v>-0.3724364601404745</v>
       </c>
       <c r="G12">
-        <v>0.2203029411662774</v>
+        <v>0.1471283506969798</v>
       </c>
       <c r="H12">
-        <v>0.3556443556443556</v>
+        <v>0.5234765234765235</v>
       </c>
     </row>
   </sheetData>

</xml_diff>